<commit_message>
Add the L2 Step 1 MOR hard-error list and correct two earlier findings.
Remove the gap-assessment row that misread the post-capping DMF wash, and restate the batch-size note using the MOR's 1.0–1.2 mmol/g substitution criterion.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/L2-GA-140020-0301.01-批注清单.xlsx
+++ b/L2-GA-140020-0301.01-批注清单.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批注清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'批注清单'!$A$1:$D$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'批注清单'!$A$1:$D$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -809,28 +809,9 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="78" customHeight="1">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>3.2.1 第 (3) 类</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>postcapping DMF wash step using Ac2O/Pyridine/DMF is replaced by direct charging</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>终版 PVP 仍是在 TJ4S-1213-R22 配制醋酐/吡啶/DMF，搅拌至少 5 min，再转入 Sy15。封端后的洗涤是 DMF，不是封端液本身。这句把封端液和封端后洗涤混在一起。请改成与终版一致的设备流向：配制在 R22，转入 Sy15；不要写成取消配制、直接投入合成釜。</t>
-        </is>
-      </c>
-    </row>
+    <row r="18" ht="78" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:D18"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>